<commit_message>
Map tambang dalam negeri pending validation
</commit_message>
<xml_diff>
--- a/templates/permohonan-belum-peraku-template.xlsx
+++ b/templates/permohonan-belum-peraku-template.xlsx
@@ -1,24 +1,43 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
-  <bookViews>
-    <workbookView xWindow="15180" yWindow="2550" windowWidth="22395" windowHeight="11295"/>
-  </bookViews>
-  <sheets>
-    <sheet sheetId="2" name="26.6.2026" state="visible" r:id="rId4"/>
-    <sheet sheetId="3" name="Unmapped" state="visible" r:id="rId5"/>
-  </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'26.6.2026'!$B1:$R84</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'26.6.2026'!$2:$5</definedName>
-  </definedNames>
-  <calcPr calcId="171027"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>Worksheets</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>2</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="2" baseType="lpstr">
+      <vt:lpstr>26.6.2026</vt:lpstr>
+      <vt:lpstr>Unmapped</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <Company/>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>16.0300</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>Wan Lee</dc:creator>
+  <cp:lastModifiedBy>Wan Lee</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-06-03T13:10:57Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-06-04T16:05:03Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="144">
   <si>
     <t>LAPORAN PERMOHONAN BANTUAN YANG BELUM DIPERAKU</t>
@@ -123,7 +142,7 @@
     <t xml:space="preserve">BANTUAN TAMBANG DAN KEPERLUAN DIRI </t>
   </si>
   <si>
-    <t>BANTUAN TAMBANG DALAM NEGERI</t>
+    <t>BANTUAN TAMBANG DAN KEPERLUAN DIRI DALAM NEGERI</t>
   </si>
   <si>
     <t>BANTUAN TAMBANG DAN KEPERLUAN DIRI LUAR NEGERI</t>
@@ -455,7 +474,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="12" x14ac:knownFonts="1">
     <font>
@@ -1199,7 +1218,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -1514,7 +1533,26 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+  <bookViews>
+    <workbookView xWindow="15180" yWindow="2550" windowWidth="22395" windowHeight="11295"/>
+  </bookViews>
+  <sheets>
+    <sheet sheetId="2" name="26.6.2026" state="visible" r:id="rId4"/>
+    <sheet sheetId="3" name="Unmapped" state="visible" r:id="rId5"/>
+  </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'26.6.2026'!$B1:$R84</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'26.6.2026'!$2:$5</definedName>
+  </definedNames>
+  <calcPr calcId="171027"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -11881,7 +11919,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>

</xml_diff>